<commit_message>
Checkpoint news scenarios, action guidance, and lean brief packets
</commit_message>
<xml_diff>
--- a/demo/templates/neoagent-v2-campaign-tracker.xlsx
+++ b/demo/templates/neoagent-v2-campaign-tracker.xlsx
@@ -676,14 +676,14 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>The planned venue is unavailable. Northstar is holding Studio B Friday and Studio C Tuesday until 4:30 PM today.</x:v>
+        <x:v>Priya has checked both replacement options. Studio B Friday and Studio C Tuesday both meet production needs. Holds expire at 4:30 PM today.</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>Choose Studio B Friday or Studio C Tuesday before the hold expires.</x:v>
+        <x:v>Reply to Priya with the preferred option. Priya will handle booking and production arrangements.</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str"/>
       <x:c r="G10" s="9" t="str">
-        <x:v>Executive replacement-date decision; venue and preferred crew will be released without it.</x:v>
+        <x:v>Awaiting only the user's Friday/Tuesday preference before the holds expire.</x:v>
       </x:c>
       <x:c r="H10" s="9" t="str">
         <x:v>EMAIL_PRIYA</x:v>

</xml_diff>